<commit_message>
Fase 1: orçamento com fornecedores reais (ML/Amazon) e links
- Pesquisa de fornecedores e precos (out/2026) com links clicaveis
- Flags: set screw M8 em ACO (nao inox); ima em disco; bucha Ø6 rara
- Ferragem consolidada em kits reais (insertos M2-M5, parafusos M3-M5)
- Secao de observacoes com a pendencia da bucha e portao da fase

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/volante/01_documentos/orçamento.xlsx
+++ b/volante/01_documentos/orçamento.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,8 +47,16 @@
       <b val="1"/>
     </font>
     <font>
+      <color rgb="000563C1"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00C00000"/>
+    </font>
+    <font>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -149,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -167,16 +175,22 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -543,17 +557,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -566,7 +580,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Compras de longo prazo. Preencha Gasto / Fornecedor / Link / Status conforme comprar. Valores previstos são estimativas (confirmar preço real).</t>
+          <t>Fornecedores e preços pesquisados em out/2026 (Mercado Livre / Amazon / Shopee) — CONFIRMAR antes de comprar, preço e estoque mudam. Preencha Gasto / Link escolhido / Status.</t>
         </is>
       </c>
     </row>
@@ -580,14 +594,14 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>⚠️ Ímã N52, nunca N35 (força bem menor).</t>
+          <t>⚠️ Ímã N52 em formato DISCO/CILINDRO (não 'bloco'); nunca N35.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>⚠️ Set screw M8 em AÇO (não inox/latão): o ímã de retorno precisa atrair aço.</t>
+          <t>⚠️ Set screw M8 em AÇO (não inox A2/A4): o ímã de retorno precisa atrair aço.</t>
         </is>
       </c>
     </row>
@@ -624,7 +638,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Link (colar)</t>
+          <t>Link (ref.)</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -650,7 +664,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Raspberry Pi Pico (RP2040), com pinos soldados</t>
+          <t>Raspberry Pi Pico H (RP2040) — pinos JÁ soldados (versão 'H')</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -662,7 +676,7 @@
         <v>80</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="E10" s="10" t="n"/>
       <c r="F10" s="9" t="inlineStr">
@@ -670,7 +684,11 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n"/>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-3181190378-raspberry-pi-pico-h-rp2040-dual-core-arm-cortex-m0-264kb-_JM</t>
+        </is>
+      </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -680,27 +698,31 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Botão tátil 12 × 12 mm</t>
+          <t>Kit 25 push button 12×12 mm (chave táctil)</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1 kit (usa 15)</t>
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E11" s="10" t="n"/>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Shopee</t>
-        </is>
-      </c>
-      <c r="G11" s="11" t="n"/>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-1757293010-kit-25-push-button-12x12-chave-tactil-capa-_JM</t>
+        </is>
+      </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -710,27 +732,31 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Diodo 1N4148</t>
+          <t>Diodo 1N4148 — kit 100 peças</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1 kit (usa 15)</t>
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E12" s="10" t="n"/>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Shopee</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="n"/>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-2030445588-diodo-de-sinal-1n4148-kit-100-pecas-_JM</t>
+        </is>
+      </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -740,19 +766,19 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Encoder rotativo EC11 (20 pulsos, com clique)</t>
+          <t>Encoder rotativo EC11 (20 pulsos, c/ clique) — pacote 10</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>5 (1 reserva)</t>
+          <t>1 pct (usa 5)</t>
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="E13" s="10" t="n"/>
       <c r="F13" s="9" t="inlineStr">
@@ -760,7 +786,11 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="G13" s="11" t="n"/>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-2936813951-encoder-rotativo-ec11-potenciometro-10-unidades-arduino-_JM</t>
+        </is>
+      </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -770,16 +800,16 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Sensor Hall linear SS49E</t>
+          <t>Sensor Hall linear SS49E — kit 5 peças</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>3 (1 reserva)</t>
+          <t>1 kit (usa 3)</t>
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D14" s="10" t="n">
         <v>25</v>
@@ -787,10 +817,14 @@
       <c r="E14" s="10" t="n"/>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Shopee</t>
-        </is>
-      </c>
-      <c r="G14" s="11" t="n"/>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-1367538567-sensor-hall-49e-oh49e-ss49e-analogico-kit-5-pecas-_JM</t>
+        </is>
+      </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -800,19 +834,19 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Protoboard 830 pontos</t>
+          <t>Kit protoboard 830 pontos + 65 jumpers (MB102)</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1 kit</t>
         </is>
       </c>
       <c r="C15" s="10" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E15" s="10" t="n"/>
       <c r="F15" s="9" t="inlineStr">
@@ -820,7 +854,11 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n"/>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kit-protoboard-830-pontos-fonte-mb102-kit-jumpers-arduino/p/MLB37389913</t>
+        </is>
+      </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -830,7 +868,7 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Kit de jumpers macho-macho</t>
+          <t>Protoboard 830 pontos — 2ª unidade</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -847,10 +885,14 @@
       <c r="E16" s="10" t="n"/>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Shopee</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="n"/>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>https://lista.mercadolivre.com.br/protoboard-830</t>
+        </is>
+      </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -860,7 +902,7 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Cabo USB-A → micro-USB (com dados)</t>
+          <t>Cabo USB-A → micro-USB com DADOS (ex.: C3Tech CB-M11)</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
@@ -877,10 +919,14 @@
       <c r="E17" s="10" t="n"/>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="n"/>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/cabo-micro-usb-1m-preto-2a-c3tech-conector-v8-cb-m11-transferencia-de-dados/p/MLB22252705</t>
+        </is>
+      </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -890,7 +936,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>B. ÍMÃS DE NEODÍMIO N52</t>
+          <t>B. ÍMÃS DE NEODÍMIO N52 (formato DISCO)</t>
         </is>
       </c>
       <c r="B18" s="6" t="n"/>
@@ -904,19 +950,19 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Ímã N52 Ø10 × 5 mm (retorno da aleta)</t>
+          <t>Ímã N52 Ø10 × 5 mm DISCO (retorno da aleta) — pacote</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1 pct (usa 2)</t>
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="E19" s="10" t="n"/>
       <c r="F19" s="9" t="inlineStr">
@@ -924,7 +970,11 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="G19" s="11" t="n"/>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>https://lista.mercadolivre.com.br/ima-de-neod%C3%ADmio-10x5mm</t>
+        </is>
+      </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -934,19 +984,19 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Ímã N52 Ø5 × 3 mm (sensor Hall)</t>
+          <t>Ímã N52 Ø5 × 3 mm DISCO (sensor Hall) — pacote</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1 pct (usa 6)</t>
         </is>
       </c>
       <c r="C20" s="10" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E20" s="10" t="n"/>
       <c r="F20" s="9" t="inlineStr">
@@ -954,7 +1004,11 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="G20" s="11" t="n"/>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>https://lista.mercadolivre.com.br/ima-neodimio-5x3</t>
+        </is>
+      </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -978,19 +1032,19 @@
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Eixo de aço Ø4 × ~44 mm (giro da aleta)</t>
+          <t>Eixo: barra redonda inox 304 Ø4 mm (cortar 2× ~44 mm)</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1 barra</t>
         </is>
       </c>
       <c r="C22" s="10" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="E22" s="10" t="n"/>
       <c r="F22" s="9" t="inlineStr">
@@ -998,7 +1052,11 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n"/>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/barra-redonda-de-inox-304--4mm-x-36-cm/up/MLBU1980168840</t>
+        </is>
+      </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -1008,7 +1066,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Bucha de bronze Ø4 × Ø6 × 4 mm</t>
+          <t>Bucha de bronze Ø4 × Ø6 × 4 mm ⚠️ ver obs. (OD6 raro)</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -1017,18 +1075,22 @@
         </is>
       </c>
       <c r="C23" s="10" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="E23" s="10" t="n"/>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Mercado Livre</t>
-        </is>
-      </c>
-      <c r="G23" s="11" t="n"/>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>https://lista.mercadolivre.com.br/bucha-bronze-sinterizado</t>
+        </is>
+      </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -1038,19 +1100,19 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Set screw M8 × 10 ponta plana (aço)</t>
+          <t>Set screw M8 × 10 ponta plana — AÇO (não inox!) DIN 913</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2 (pct)</t>
         </is>
       </c>
       <c r="C24" s="10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E24" s="10" t="n"/>
       <c r="F24" s="9" t="inlineStr">
@@ -1058,7 +1120,11 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n"/>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-3273317985-parafuso-allen-sem-cabeca-com-rebaixo-m8-x-10mm-20-pecas-_JM</t>
+        </is>
+      </c>
       <c r="H24" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -1068,27 +1134,31 @@
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Inserto roscado M3 a quente</t>
+          <t>Kit insertos latão a quente M2–M5 (cobre M3 e M4)</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>~10</t>
+          <t>1 kit</t>
         </is>
       </c>
       <c r="C25" s="10" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E25" s="10" t="n"/>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Shopee</t>
-        </is>
-      </c>
-      <c r="G25" s="11" t="n"/>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/inser%C3%A7%C3%B5es-impress%C3%A3o-serrilhadas-rosqueado-componentes/dp/B0CY2HGFB8</t>
+        </is>
+      </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -1098,27 +1168,31 @@
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Inserto roscado M4 a quente</t>
+          <t>Kit parafusos allen M3/M4/M5 + porcas (cobre M3×8, M4, M5)</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>~4</t>
+          <t>1 kit</t>
         </is>
       </c>
       <c r="C26" s="10" t="n">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="E26" s="10" t="n"/>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Shopee</t>
-        </is>
-      </c>
-      <c r="G26" s="11" t="n"/>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Parafusos-Allen-Cabe%C3%A7a-Redonda-Porcas/dp/B0FPZ2M1YF</t>
+        </is>
+      </c>
       <c r="H26" s="9" t="inlineStr">
         <is>
           <t>Pendente</t>
@@ -1126,226 +1200,171 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>Parafuso M3 × 8</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>~10</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="D27" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="E27" s="10" t="n"/>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>Shopee</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="n"/>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>Parafuso M4 × ~10</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>~4</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="E28" s="10" t="n"/>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>Shopee</t>
-        </is>
-      </c>
-      <c r="G28" s="11" t="n"/>
-      <c r="H28" s="9" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL FASE 1</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="13">
+        <f>SUM(C10:C26)</f>
+        <v/>
+      </c>
+      <c r="D27" s="13">
+        <f>SUM(D10:D26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="13">
+        <f>SUM(E10:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="12" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>Parafuso M5 (interface base 6 furos × 70 mm)</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="D29" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="E29" s="10" t="n"/>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>Mercado Livre</t>
-        </is>
-      </c>
-      <c r="G29" s="11" t="n"/>
-      <c r="H29" s="9" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>❌ NÃO COMPRAR AGORA (dependem da maquete / Fase 7)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Porcas M3 / M4 / M5 (kit)</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>1 kit</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="D30" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="E30" s="10" t="n"/>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>Mercado Livre</t>
-        </is>
-      </c>
-      <c r="G30" s="11" t="n"/>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>12 botões de painel (10× Ø16 + 2× Ø19) — corpo ≤ 25 mm atrás da placa</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="n"/>
+      <c r="C30" s="16" t="n"/>
+      <c r="D30" s="16" t="n"/>
+      <c r="E30" s="16" t="n"/>
+      <c r="F30" s="16" t="n"/>
+      <c r="G30" s="16" t="n"/>
+      <c r="H30" s="17" t="inlineStr">
+        <is>
+          <t>após a maquete (Fase 2)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>TOTAL FASE 1</t>
-        </is>
-      </c>
-      <c r="B31" s="12" t="n"/>
-      <c r="C31" s="13">
-        <f>SUM(C10:C30)</f>
-        <v/>
-      </c>
-      <c r="D31" s="13">
-        <f>SUM(D10:D30)</f>
-        <v/>
-      </c>
-      <c r="E31" s="13">
-        <f>SUM(E10:E30)</f>
-        <v/>
-      </c>
-      <c r="F31" s="12" t="n"/>
-      <c r="G31" s="12" t="n"/>
-      <c r="H31" s="12" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="14" t="inlineStr">
-        <is>
-          <t>❌ NÃO COMPRAR AGORA (dependem da maquete / Fase 7)</t>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>4 knobs Ø26</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="n"/>
+      <c r="C31" s="16" t="n"/>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="16" t="n"/>
+      <c r="F31" s="16" t="n"/>
+      <c r="G31" s="16" t="n"/>
+      <c r="H31" s="17" t="inlineStr">
+        <is>
+          <t>após a maquete (Fase 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>Base Moza R3 + adaptador quick release</t>
+        </is>
+      </c>
+      <c r="B32" s="16" t="n"/>
+      <c r="C32" s="16" t="n"/>
+      <c r="D32" s="16" t="n"/>
+      <c r="E32" s="16" t="n"/>
+      <c r="F32" s="16" t="n"/>
+      <c r="G32" s="16" t="n"/>
+      <c r="H32" s="17" t="inlineStr">
+        <is>
+          <t>Fase 7</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="inlineStr">
-        <is>
-          <t>12 botões de painel (10× Ø16 + 2× Ø19) — corpo ≤ 25 mm atrás da placa</t>
-        </is>
-      </c>
-      <c r="B34" s="16" t="n"/>
-      <c r="C34" s="16" t="n"/>
-      <c r="D34" s="16" t="n"/>
-      <c r="E34" s="16" t="n"/>
-      <c r="F34" s="16" t="n"/>
-      <c r="G34" s="16" t="n"/>
-      <c r="H34" s="17" t="inlineStr">
-        <is>
-          <t>após a maquete (Fase 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
-        <is>
-          <t>4 knobs Ø26</t>
-        </is>
-      </c>
-      <c r="B35" s="16" t="n"/>
-      <c r="C35" s="16" t="n"/>
-      <c r="D35" s="16" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="16" t="n"/>
-      <c r="G35" s="16" t="n"/>
-      <c r="H35" s="17" t="inlineStr">
-        <is>
-          <t>após a maquete (Fase 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="15" t="inlineStr">
-        <is>
-          <t>Base Moza R3 + adaptador quick release</t>
-        </is>
-      </c>
-      <c r="B36" s="16" t="n"/>
-      <c r="C36" s="16" t="n"/>
-      <c r="D36" s="16" t="n"/>
-      <c r="E36" s="16" t="n"/>
-      <c r="F36" s="16" t="n"/>
-      <c r="G36" s="16" t="n"/>
-      <c r="H36" s="17" t="inlineStr">
-        <is>
-          <t>Fase 7</t>
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>OBSERVAÇÕES</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>• Bucha de bronze: a medida Ø4×Ø6×4 (OD 6 mm) quase não existe no varejo; o comum é Ø4×Ø8×8 (OD 8 mm). Como o CAD é paramétrico, o ideal é ajustar o furo do carregador/suporte para a bucha Ø8 disponível — decidir com quem mantém o CAD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>• Eixo Ø4: a barra de inox serve (o eixo NÃO precisa ser magnético, só o set screw M8). Cortar 2 pedaços de ~44 mm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>• Total subiu vs. estimativa inicial porque ímãs/parafusos/insertos são vendidos em PACOTES/KITS (sobra reserva).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="19" t="inlineStr">
+        <is>
+          <t>• Shopee costuma ter os itens de eletrônica mais baratos — vale comparar antes de fechar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>• Portão da Fase 1: receber e conferir item por item; medir ímãs e eixo com paquímetro.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="15">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A36:H36"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A37:H37"/>
     <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H10 H11 H12 H13 H14 H15 H16 H17 H19 H20 H22 H23 H24 H25 H26 H27 H28 H29 H30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H10 H11 H12 H13 H14 H15 H16 H17 H19 H20 H22 H23 H24 H25 H26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Comprado,Recebido/Conferido"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId15"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>